<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.002-01 La cabane de biscuits de Nino
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.002-01.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.002-01.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine le dimanche</t>
+          <t>cuisine le dimanche, casserole de cuivre, zestes, coquille d'œuf</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nino, Aniss, papa</t>
+          <t>Nino, Aniss, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino veut une cabane de biscuits au citron. Aniss arrive. Un rire commence. Papa dit : le corps n'est pas une blague. Ils bâtissent le toit, ensemble.</t>
+          <t>Une goutte de beurre saute dans le cuivre. Sur le bord, un éclat de cuivre brille. Nino veut une cabane de biscuits, maintenant. Aniss arrive. Le tablier glisse autrement. Un rire commence. Aniss se tait. Le toit tombe. Nino refuse de foncer. Ils tiennent les murs, à deux. Merci vécu. Un biscuit rond trop vite. L'éclat de cuivre tient sur le bord.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La casserole de cuivre fait tic sur le feu. Des zestes de citron brillent sur la planche. Une coquille d'œuf est encore collée. Ça sent le beurre tiède. Le carrelage est froid sous les pieds. Un torchon à carreaux pend. Tu as vu le citron, Nino ? Oui, papa. Il pique le nez. On fait des biscuits. En ce moment, Nino pose un biscuit plat. Il en pose un autre à côté. Je veux une cabane. Une cabane de biscuits. Avec un toit ? Oui. Un grand toit. Aniss arrive. Il enlève ses chaussures. Ses chaussettes sont jaunes. Papa tend deux tabliers. Le tablier d'Aniss tombe autrement. Aniss a un corps plus rond. Nino a un corps plus mince. Un petit rire commence. Le corps n'est pas une blague. On joue. On cuisine. Nino ferme la bouche. Il hoche la tête. On fait la cabane. Oui. La pâte est froide et un peu collante. Elle sent le citron. Un peu de farine reste sur la planche. Aniss, tu tiens le mur ? Je le tiens. Tout doux, les murs.</t>
+          <t>Une goutte de beurre saute dans le cuivre. Elle fait tic, chaud et rond. Ça saute, papa ! Tu l'entends, dans la casserole ? Oui, un petit tic. La casserole de cuivre tient sur le feu. Sur le bord, un éclat de cuivre brille. Il brille, maman. Tu le vois, sur le cuivre ? Oui, un petit point. Des zestes de citron piquent l'air. Une coquille d'œuf reste collée au bol. Ça sent le beurre, un peu tiède. Ça sent le citron. On fait des biscuits, Nino ? Oui, papa. Le carrelage est froid, sous les pieds. Il pique un peu. Un torchon à carreaux pend près du feu. Je veux une cabane, maintenant ! Une cabane de biscuits ? Oui, avec un grand toit. En ce moment, Nino pose un biscuit plat. Il en pose un autre trop vite. Le biscuit penche, puis se redresse. Le mur, papa ! Il tient, Nino ? Presque. Aniss arrive près de la table. Il enlève ses chaussures, sans un mot. Ses chaussettes sont jaunes, un peu épaisses. Aniss ! J'arrive. Tes chaussettes sont jaunes, Aniss ? Oui. Papa tend deux tabliers. Le tablier d'Aniss glisse plus bas. Il tombe drôle ! Un rire commence dans la bouche de Nino. Aniss ne dit rien. Le sourire d'Aniss disparaît. Tu tiens le mur, maintenant ! Aniss recule d'un pas. Non. Oh. Nino pose le toit trop vite, tout seul. Le toit glisse, puis tombe. Il tombe ! Oh. L'éclat de cuivre tremble, puis tient. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Nino ? Oui, papa. Tes mains sont collantes, Nino ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La casserole de cuivre fait tic sur le feu. Des zestes de citron brillent sur la planche. Une coquille d'œuf est encore collée. Ça sent le beurre tiède. Le carrelage est froid sous les pieds. Un torchon à carreaux pend. Tu as vu le citron, Nino ? Oui, papa. Il pique le nez. On fait des biscuits. En ce moment, Nino pose un biscuit plat. Il en pose un autre à côté. Je veux une cabane. Une cabane de biscuits. Avec un toit ? Oui. Un grand toit. Aniss arrive. Il enlève ses chaussures. Ses chaussettes sont jaunes. Papa tend deux tabliers. Le tablier d'Aniss tombe autrement. Aniss a un corps plus rond. Nino a un corps plus mince. Un petit rire commence. Le corps n'est pas une blague. On joue. On cuisine. Nino ferme la bouche. Il hoche la tête. On fait la cabane. Oui. La pâte est froide et un peu collante. Elle sent le citron. Un peu de farine reste sur la planche. Aniss, tu tiens le mur ? Je le tiens. Tout doux, les murs.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte de beurre saute dans le cuivre. Elle fait tic, chaud et rond. Ça saute, papa ! Tu l'entends, dans la casserole ? Oui, un petit tic. La casserole de cuivre tient sur le feu. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de cuivre&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, sur le cuivre ? Oui, un petit point. Des zestes de citron piquent l'air. Une coquille d'œuf reste collée au bol. Ça sent le beurre, un peu tiède. Ça sent le citron. On fait des biscuits, Nino ? Oui, papa. Le carrelage est froid, sous les pieds. Il pique un peu. Un torchon à carreaux pend près du feu. Je veux une cabane, maintenant ! Une cabane de biscuits ? Oui, avec un grand toit. En ce moment, Nino pose un biscuit plat. Il en pose un autre trop vite. Le biscuit penche, puis se redresse. Le mur, papa ! Il tient, Nino ? Presque. Aniss arrive près de la table. Il enlève ses chaussures, sans un mot. Ses chaussettes sont jaunes, un peu épaisses. Aniss ! J'arrive. Tes chaussettes sont jaunes, Aniss ? Oui. Papa tend deux tabliers. Le tablier d'Aniss glisse plus bas. Il tombe drôle ! Un rire commence dans la bouche de Nino. Aniss ne dit rien. Le sourire d'Aniss disparaît. Tu tiens le mur, maintenant ! Aniss recule d'un pas. Non. Oh. Nino pose le toit trop vite, tout seul. Le toit glisse, puis tombe. Il tombe ! Oh. L'éclat de cuivre tremble, puis tient. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Nino ? Oui, papa. Tes mains sont collantes, Nino ? Un peu, maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Il pleut un peu. Jules est à la maison. Papa prépare de la pâte à biscuits. Adam arrive. Il enlève ses chaussures. Papa dit : on fait des biscuits ensemble. Jules met un tablier. Adam met un tablier. Les tabliers tombent un peu différemment. Adam a un ventre plus rond. Jules a des bras plus minces. Jules regarde. Il ouvre la bouche. Un petit rire commence. Papa parle tout de suite. Papa dit : le &lt;emphasis&gt;corps&lt;/emphasis&gt; n'est pas une blague. On joue. On cuisine. On reste gentils. Jules ferme la bouche. Il hoche la tête. Adam prend un emporte-pièce étoile. Jules prend un emporte-pièce lune. Ils posent les formes dans la pâte. Papa dit encore : le corps n'est pas une blague. L'amitié ne dépend pas de la forme. On peut jouer. La pâte est froide et douce. Jules étale un morceau. Adam étale un morceau. Ils se passent la farine. Un nuage blanc monte. Ils sourient. Papa met les biscuits au chaud. En attendant, ils font une tour de bols. Adam tient la base. Jules pose le petit bol. La tour tient. Papa dit : vous jouez. C'est ça. On ne commente pas le corps pour rabaisser. On joue. Les biscuits sentent le beurre. Papa les pose à refroidir. Jules offre une étoile à Adam. Adam offre une lune à Jules. Ils croquent. C'est sucré. Papa dit : le corps n'est pas une blague. On joue, et on mange ensemble. [pause]</t>
+          <t>Une goutte de beurre saute dans le cuivre. Elle fait tic, chaud et rond. Ça saute, papa ! Tu l'entends, dans la casserole ? Oui, un petit tic. La casserole de cuivre tient sur le feu. Sur le bord, un &lt;emphasis&gt;éclat de cuivre&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, sur le cuivre ? Oui, un petit point. Des zestes de citron piquent l'air. Une coquille d'œuf reste collée au bol. Ça sent le beurre, un peu tiède. Ça sent le citron. On fait des biscuits, Nino ? Oui, papa. Le carrelage est froid, sous les pieds. Il pique un peu. Un torchon à carreaux pend près du feu. Je veux une cabane, maintenant ! Une cabane de biscuits ? Oui, avec un grand toit. En ce moment, Nino pose un biscuit plat. Il en pose un autre trop vite. Le biscuit penche, puis se redresse. Le mur, papa ! Il tient, Nino ? Presque. Aniss arrive près de la table. Il enlève ses chaussures, sans un mot. Ses chaussettes sont jaunes, un peu épaisses. Aniss ! J'arrive. Tes chaussettes sont jaunes, Aniss ? Oui. Papa tend deux tabliers. Le tablier d'Aniss glisse plus bas. Il tombe drôle ! Un rire commence dans la bouche de Nino. Aniss ne dit rien. Le sourire d'Aniss disparaît. Tu tiens le mur, maintenant ! Aniss recule d'un pas. Non. Oh. Nino pose le toit trop vite, tout seul. Le toit glisse, puis tombe. Il tombe ! Oh. L'éclat de cuivre tremble, puis tient. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Nino ? Oui, papa. Tes mains sont collantes, Nino ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>éclat de cuivre</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,47 +1321,76 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_cabane_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La casserole de cuivre fait tic sur le feu.
-narrateur|Des zestes de citron brillent sur la planche.
-narrateur|Une coquille d'œuf est encore collée.
-narrateur|Ça sent le beurre tiède.
-narrateur|Le carrelage est froid sous les pieds.
-narrateur|Un torchon à carreaux pend.
-papa|Tu as vu le citron, Nino ?
+          <t>narrateur|Une goutte de beurre saute dans le cuivre.
+narrateur|Elle fait tic, chaud et rond.
+enfant-m|Ça saute, papa !
+papa|Tu l'entends, dans la casserole ?
+enfant-m|Oui, un petit tic.
+narrateur|La casserole de cuivre tient sur le feu.
+narrateur|Sur le bord, un éclat de cuivre brille.
+enfant-m|Il brille, maman.
+maman|Tu le vois, sur le cuivre ?
+enfant-m|Oui, un petit point.
+narrateur|Des zestes de citron piquent l'air.
+narrateur|Une coquille d'œuf reste collée au bol.
+narrateur|Ça sent le beurre, un peu tiède.
+enfant-m|Ça sent le citron.
+papa|On fait des biscuits, Nino ?
 enfant-m|Oui, papa.
-enfant-m|Il pique le nez.
-papa|On fait des biscuits.
+maman|Le carrelage est froid, sous les pieds.
+enfant-m|Il pique un peu.
+narrateur|Un torchon à carreaux pend près du feu.
+enfant-m|Je veux une cabane, maintenant !
+papa|Une cabane de biscuits ?
+enfant-m|Oui, avec un grand toit.
 narrateur|En ce moment, Nino pose un biscuit plat.
-narrateur|Il en pose un autre à côté.
-enfant-m|Je veux une cabane.
-enfant-m|Une cabane de biscuits.
-papa|Avec un toit ?
-enfant-m|Oui.
-enfant-m|Un grand toit.
-narrateur|Aniss arrive.
-narrateur|Il enlève ses chaussures.
-narrateur|Ses chaussettes sont jaunes.
+narrateur|Il en pose un autre trop vite.
+narrateur|Le biscuit penche, puis se redresse.
+enfant-m|Le mur, papa !
+papa|Il tient, Nino ?
+enfant-m|Presque.
+narrateur|Aniss arrive près de la table.
+narrateur|Il enlève ses chaussures, sans un mot.
+narrateur|Ses chaussettes sont jaunes, un peu épaisses.
+enfant-m|Aniss !
+copain|J'arrive.
+maman|Tes chaussettes sont jaunes, Aniss ?
+copain|Oui.
 narrateur|Papa tend deux tabliers.
-narrateur|Le tablier d'Aniss tombe autrement.
-narrateur|Aniss a un corps plus rond.
-narrateur|Nino a un corps plus mince.
-narrateur|Un petit rire commence.
-papa|Le corps n'est pas une blague.
-papa|On joue.
-papa|On cuisine.
-narrateur|Nino ferme la bouche.
-narrateur|Il hoche la tête.
-enfant-m|On fait la cabane.
-copain|Oui.
-narrateur|La pâte est froide et un peu collante.
-narrateur|Elle sent le citron.
-narrateur|Un peu de farine reste sur la planche.
-enfant-m|Aniss, tu tiens le mur ?
-copain|Je le tiens.
-papa|Tout doux, les murs.</t>
+narrateur|Le tablier d'Aniss glisse plus bas.
+enfant-m|Il tombe drôle !
+narrateur|Un rire commence dans la bouche de Nino.
+narrateur|Aniss ne dit rien.
+narrateur|Le sourire d'Aniss disparaît.
+enfant-m|Tu tiens le mur, maintenant !
+narrateur|Aniss recule d'un pas.
+copain|Non.
+enfant-m|Oh.
+narrateur|Nino pose le toit trop vite, tout seul.
+narrateur|Le toit glisse, puis tombe.
+enfant-m|Il tombe !
+copain|Oh.
+narrateur|L'éclat de cuivre tremble, puis tient.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Aniss, Nino ?
+enfant-m|Oui, papa.
+maman|Tes mains sont collantes, Nino ?
+enfant-m|Un peu, maman.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>casserole,feu</t>
         </is>
       </c>
     </row>
@@ -1393,12 +1422,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le corps n'est pas une blague. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;corps&lt;/emphasis&gt; n'est pas une blague. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le &lt;emphasis&gt;corps&lt;/emphasis&gt; n'est pas une blague. Que fait-on ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le &lt;emphasis&gt;corps&lt;/emphasis&gt; n'est pas une blague. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1461,7 +1490,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1472,7 +1501,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1487,11 +1516,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1502,23 +1531,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1533,17 +1562,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=on_joue_on_ne_rit_pas_du_corps; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1576,17 +1605,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Ils collent deux biscuits debout. Un peu de pâte sert de colle. Nino pose le grand biscuit du toit. Le toit glisse. Il tombe. Encore. On recommence, tout doux. Aniss tient les murs. Nino pose le toit plus lentement. Cette fois, ça tient. Une porte. Une fenêtre. Ils percent un petit trou. Le citron sent plus fort. Bravo, Nino. Tu as posé le toit. Vous jouez. Papa glisse un sucre sur le toit. Une cheminée. Elle est petite. Elle est belle. Nino tapote le toit du doigt. Le biscuit tient. L'amitié ne dépend pas de la forme. On joue.</t>
+          <t>Nino veut le toit, tout de suite. Je le pose, maintenant ! Il avance trop vite vers les murs. Les mots se bousculent dans sa bouche. Non. Aniss reste un peu plus loin. Oh. Le sourire ne revient pas. Nino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe les biscuits, un instant. Il écoute le tic du cuivre. Tu veux le toit avec Aniss ? Papa reste à la même hauteur. Tu tiens les murs ? Aniss ne dit rien, d'abord. Il pose les mains sur les biscuits. Je les tiens. D'accord. Merci, Nino. Papa a vu les deux, près de la table. La pâte colle un peu, sous les doigts. Elle est froide. Nino pose le toit, sans se presser. Aniss tient les murs, plus large. Le toit reste, cette fois. Il tient ! Oui. Tu le vois, le toit ? Oui, papa. Une porte, Nino ? Un petit trou. Ils percent un trou, tout près. Le citron sent plus fort. Une fenêtre. Oui, une fenêtre. Le ventre de Nino se desserre. Les épaules se relèvent un peu. On reste à la table ? Oui. Tes mains sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Ils collent deux biscuits debout. Un peu de pâte sert de colle. Nino pose le grand biscuit du toit. Le toit glisse. Il tombe. Encore. On recommence, tout doux. Aniss tient les murs. Nino pose le toit plus lentement. Cette fois, ça tient. Une porte. Une fenêtre. Ils percent un petit trou. Le citron sent plus fort. Bravo, Nino. Tu as posé le toit. Vous jouez. Papa glisse un sucre sur le toit. Une cheminée. Elle est petite. Elle est belle. Nino tapote le toit du doigt. Le biscuit tient. L'amitié ne dépend pas de la forme. On joue.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino veut le toit, tout de suite. Je le pose, maintenant ! Il avance trop vite vers les &lt;emphasis level="moderate"&gt;murs&lt;/emphasis&gt;. Les mots se bousculent dans sa bouche. Non. Aniss reste un peu plus loin. Oh. Le sourire ne revient pas. Nino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe les biscuits, un instant. Il écoute le tic du cuivre. Tu veux le toit avec Aniss ? Papa reste à la même hauteur. Tu tiens les murs ? Aniss ne dit rien, d'abord. Il pose les mains sur les biscuits. Je les tiens. D'accord. Merci, Nino. Papa a vu les deux, près de la table. La pâte colle un peu, sous les doigts. Elle est froide. Nino pose le toit, sans se presser. Aniss tient les murs, plus large. Le toit reste, cette fois. Il tient ! Oui. Tu le vois, le toit ? Oui, papa. Une porte, Nino ? Un petit trou. Ils percent un trou, tout près. Le citron sent plus fort. Une fenêtre. Oui, une fenêtre. Le ventre de Nino se desserre. Les épaules se relèvent un peu. On reste à la table ? Oui. Tes mains sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Jules a entendu papa. Le &lt;emphasis&gt;corps&lt;/emphasis&gt; n'est pas une blague. Jules et Adam ont joué. Ils ont fait des biscuits. [pause]</t>
+          <t>Nino veut le toit, tout de suite. Je le pose, maintenant ! Il avance trop vite vers les &lt;emphasis&gt;murs&lt;/emphasis&gt;. Les mots se bousculent dans sa bouche. Non. Aniss reste un peu plus loin. Oh. Le sourire ne revient pas. Nino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe les biscuits, un instant. Il écoute le tic du cuivre. Tu veux le toit avec Aniss ? Papa reste à la même hauteur. Tu tiens les murs ? Aniss ne dit rien, d'abord. Il pose les mains sur les biscuits. Je les tiens. D'accord. Merci, Nino. Papa a vu les deux, près de la table. La pâte colle un peu, sous les doigts. Elle est froide. Nino pose le toit, sans se presser. Aniss tient les murs, plus large. Le toit reste, cette fois. Il tient ! Oui. Tu le vois, le toit ? Oui, papa. Une porte, Nino ? Un petit trou. Ils percent un trou, tout près. Le citron sent plus fort. Une fenêtre. Oui, une fenêtre. Le ventre de Nino se desserre. Les épaules se relèvent un peu. On reste à la table ? Oui. Tes mains sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1633,7 +1662,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1641,10 +1670,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1667,30 +1696,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>murs</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1699,10 +1728,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1715,36 +1744,59 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=ils_tiennent_les_murs_a_deux; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Ils collent deux biscuits debout.
-narrateur|Un peu de pâte sert de colle.
-narrateur|Nino pose le grand biscuit du toit.
-narrateur|Le toit glisse.
-enfant-m|Il tombe.
-copain|Encore.
-papa|On recommence, tout doux.
-narrateur|Aniss tient les murs.
-narrateur|Nino pose le toit plus lentement.
-narrateur|Cette fois, ça tient.
-enfant-m|Une porte.
+          <t>narrateur|Nino veut le toit, tout de suite.
+enfant-m|Je le pose, maintenant !
+narrateur|Il avance trop vite vers les murs.
+narrateur|Les mots se bousculent dans sa bouche.
+copain|Non.
+narrateur|Aniss reste un peu plus loin.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Nino refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe les biscuits, un instant.
+narrateur|Il écoute le tic du cuivre.
+papa|Tu veux le toit avec Aniss ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Tu tiens les murs ?
+narrateur|Aniss ne dit rien, d'abord.
+narrateur|Il pose les mains sur les biscuits.
+copain|Je les tiens.
+enfant-m|D'accord.
+papa|Merci, Nino.
+narrateur|Papa a vu les deux, près de la table.
+maman|La pâte colle un peu, sous les doigts.
+enfant-m|Elle est froide.
+narrateur|Nino pose le toit, sans se presser.
+narrateur|Aniss tient les murs, plus large.
+narrateur|Le toit reste, cette fois.
+enfant-m|Il tient !
+copain|Oui.
+papa|Tu le vois, le toit ?
+enfant-m|Oui, papa.
+maman|Une porte, Nino ?
+enfant-m|Un petit trou.
+narrateur|Ils percent un trou, tout près.
+narrateur|Le citron sent plus fort.
 copain|Une fenêtre.
-narrateur|Ils percent un petit trou.
-narrateur|Le citron sent plus fort.
-papa|Bravo, Nino.
-papa|Tu as posé le toit.
-papa|Vous jouez.
-narrateur|Papa glisse un sucre sur le toit.
-papa|Une cheminée.
-enfant-m|Elle est petite.
-copain|Elle est belle.
-narrateur|Nino tapote le toit du doigt.
-narrateur|Le biscuit tient.
-papa|L'amitié ne dépend pas de la forme.
-papa|On joue.</t>
+enfant-m|Oui, une fenêtre.
+narrateur|Le ventre de Nino se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste à la table ?
+enfant-m|Oui.
+maman|Tes mains sont au chaud ?
+enfant-m|Un peu, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pate,biscuit</t>
         </is>
       </c>
     </row>
@@ -1771,17 +1823,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On goûte la porte ? Oui. Nino casse un tout petit bout. Aniss casse l'autre bout. C'est sucré. Et citron. Tu as fini de goûter ? Oui, papa. Il reste les murs et le toit. La casserole ne fait plus tic. On essuie la planche ? Oui. Nino tient le torchon. Aniss tient l'autre bout. Le citron brille encore un peu. La cabane reste au milieu de la table.</t>
+          <t>Nino prend un biscuit plus rond. Il veut une cheminée, tout de suite. Une cheminée, maintenant ! Il regarde le tablier d'Aniss, trop longtemps. Un rire revient dans sa bouche. Attends. Aniss lâche les murs. La cabane penche vers la table. Ça tombe ! Nino avance les mains, trop vite. Puis il s'arrête net. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la cabane, un instant. Il écoute le tic du cuivre. Sur le bord, un éclat de cuivre luit. Là, sur le bord. Tu tiens, Aniss ? Aniss ne dit rien. Il reprend les murs, sans parler. Oui. Nino pose le biscuit rond, sans se presser. Papa glisse un sucre sur le toit. Une petite cheminée ? Elle est petite. Elle est belle. Un peu de sucre reste collé. Il tient. Tu restes un peu ? Oui, papa. La casserole ne fait plus tic. On la laisse ? Oui, sur le feu éteint. La cabane sent le citron. Elle colle aux doigts. Comme la pâte, oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On goûte la porte ? Oui. Nino casse un tout petit bout. Aniss casse l'autre bout. C'est sucré. Et citron. Tu as fini de goûter ? Oui, papa. Il reste les murs et le toit. La casserole ne fait plus tic. On essuie la planche ? Oui. Nino tient le torchon. Aniss tient l'autre bout. Le citron brille encore un peu. La cabane reste au milieu de la table.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino prend un biscuit plus rond. Il veut une cheminée, tout de suite. Une cheminée, maintenant ! Il regarde le tablier d'Aniss, trop longtemps. Un rire revient dans sa bouche. Attends. Aniss lâche les murs. La cabane penche vers la table. Ça tombe ! Nino avance les mains, trop vite. Puis il s'arrête net. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la cabane, un instant. Il écoute le tic du cuivre. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de cuivre&lt;/emphasis&gt; luit. Là, sur le bord. Tu tiens, Aniss ? Aniss ne dit rien. Il reprend les murs, sans parler. Oui. Nino pose le biscuit rond, sans se presser. Papa glisse un sucre sur le toit. Une petite cheminée ? Elle est petite. Elle est belle. Un peu de sucre reste collé. Il tient. Tu restes un peu ? Oui, papa. La casserole ne fait plus tic. On la laisse ? Oui, sur le feu éteint. La cabane sent le citron. Elle colle aux doigts. Comme la pâte, oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>La pluie s'arrête. Papa ouvre un peu la fenêtre. L'air sent le beurre. Jules range un bol. Adam range une cuillère. Ils se disent merci. [pause]</t>
+          <t>Nino prend un biscuit plus rond. Il veut une cheminée, tout de suite. Une cheminée, maintenant ! Il regarde le tablier d'Aniss, trop longtemps. Un rire revient dans sa bouche. Attends. Aniss lâche les murs. La cabane penche vers la table. Ça tombe ! Nino avance les mains, trop vite. Puis il s'arrête net. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la cabane, un instant. Il écoute le tic du cuivre. Sur le bord, un &lt;emphasis&gt;éclat de cuivre&lt;/emphasis&gt; luit. Là, sur le bord. Tu tiens, Aniss ? Aniss ne dit rien. Il reprend les murs, sans parler. Oui. Nino pose le biscuit rond, sans se presser. Papa glisse un sucre sur le toit. Une petite cheminée ? Elle est petite. Elle est belle. Un peu de sucre reste collé. Il tient. Tu restes un peu ? Oui, papa. La casserole ne fait plus tic. On la laisse ? Oui, sur le feu éteint. La cabane sent le citron. Elle colle aux doigts. Comme la pâte, oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1828,7 +1880,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1836,10 +1888,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1860,28 +1912,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cuivre</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1890,10 +1946,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1904,25 +1960,55 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_retrouve_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>papa|On goûte la porte ?
-enfant-m|Oui.
-narrateur|Nino casse un tout petit bout.
-narrateur|Aniss casse l'autre bout.
-enfant-m|C'est sucré.
-copain|Et citron.
-papa|Tu as fini de goûter ?
+          <t>narrateur|Nino prend un biscuit plus rond.
+narrateur|Il veut une cheminée, tout de suite.
+enfant-m|Une cheminée, maintenant !
+narrateur|Il regarde le tablier d'Aniss, trop longtemps.
+narrateur|Un rire revient dans sa bouche.
+copain|Attends.
+narrateur|Aniss lâche les murs.
+narrateur|La cabane penche vers la table.
+enfant-m|Ça tombe !
+narrateur|Nino avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Nino refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe la cabane, un instant.
+narrateur|Il écoute le tic du cuivre.
+narrateur|Sur le bord, un éclat de cuivre luit.
+enfant-m|Là, sur le bord.
+enfant-m|Tu tiens, Aniss ?
+narrateur|Aniss ne dit rien.
+narrateur|Il reprend les murs, sans parler.
+copain|Oui.
+narrateur|Nino pose le biscuit rond, sans se presser.
+narrateur|Papa glisse un sucre sur le toit.
+maman|Une petite cheminée ?
+enfant-m|Elle est petite.
+copain|Elle est belle.
+narrateur|Un peu de sucre reste collé.
+enfant-m|Il tient.
+papa|Tu restes un peu ?
 enfant-m|Oui, papa.
-narrateur|Il reste les murs et le toit.
-narrateur|La casserole ne fait plus tic.
-papa|On essuie la planche ?
-copain|Oui.
-narrateur|Nino tient le torchon.
-narrateur|Aniss tient l'autre bout.
-narrateur|Le citron brille encore un peu.
-narrateur|La cabane reste au milieu de la table.</t>
+maman|La casserole ne fait plus tic.
+enfant-m|On la laisse ?
+papa|Oui, sur le feu éteint.
+narrateur|La cabane sent le citron.
+enfant-m|Elle colle aux doigts.
+maman|Comme la pâte, oui.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>sucre,biscuit</t>
         </is>
       </c>
     </row>
@@ -1949,17 +2035,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>On a fait une cabane. Le toit est resté. Vous avez joué. La cuisine sent le citron.</t>
+          <t>Ils restent près de la table. Maman essuie un peu de farine. On a fait une cabane, papa. Tu la vois, toi ? Oui, au milieu. On est bien, ici. Nino tapote le toit du doigt. Il a une trace de sucre. Tu la vois, la trace ? Oui, maman. Le toit est resté, Nino. Oui, avec Aniss. Le toit est resté. Ça sent le beurre, un peu tiède. Et le citron, maman. Oui, dans l'air. La coquille d'œuf n'est plus au bol. Un éclat de cuivre tient sur le bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>On a fait une cabane. Le toit est resté. Vous avez joué. La cuisine sent le citron.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. Maman essuie un peu de farine. On a fait une cabane, papa. Tu la vois, toi ? Oui, au milieu. On est bien, ici. Nino tapote le toit du doigt. Il a une trace de sucre. Tu la vois, la trace ? Oui, maman. Le toit est resté, Nino. Oui, avec Aniss. Le toit est resté. Ça sent le beurre, un peu tiède. Et le citron, maman. Oui, dans l'air. La coquille d'œuf n'est plus au bol. Un &lt;emphasis level="moderate"&gt;éclat de cuivre&lt;/emphasis&gt; tient sur le bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. Maman essuie un peu de farine. On a fait une cabane, papa. Tu la vois, toi ? Oui, au milieu. On est bien, ici. Nino tapote le toit du doigt. Il a une trace de sucre. Tu la vois, la trace ? Oui, maman. Le toit est resté, Nino. Oui, avec Aniss. Le toit est resté. Ça sent le beurre, un peu tiède. Et le citron, maman. Oui, dans l'air. La coquille d'œuf n'est plus au bol. Un &lt;emphasis&gt;éclat de cuivre&lt;/emphasis&gt; tient sur le bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2006,7 +2092,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2014,10 +2100,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2026,12 +2112,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2040,17 +2126,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cuivre</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2059,11 +2149,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2072,27 +2162,50 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bord; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|On a fait une cabane.
+          <t>narrateur|Ils restent près de la table.
+narrateur|Maman essuie un peu de farine.
+enfant-m|On a fait une cabane, papa.
+papa|Tu la vois, toi ?
+enfant-m|Oui, au milieu.
+maman|On est bien, ici.
+narrateur|Nino tapote le toit du doigt.
+enfant-m|Il a une trace de sucre.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|Le toit est resté, Nino.
+enfant-m|Oui, avec Aniss.
 copain|Le toit est resté.
-papa|Vous avez joué.
-narrateur|La cuisine sent le citron.</t>
+narrateur|Ça sent le beurre, un peu tiède.
+enfant-m|Et le citron, maman.
+maman|Oui, dans l'air.
+narrateur|La coquille d'œuf n'est plus au bol.
+narrateur|Un éclat de cuivre tient sur le bord.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>cuivre</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2198,6 +2311,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>